<commit_message>
BA: Session 19.10.2026 -- Testdurchlaeufe fertig vorbereitet, Excel-Templates, Druckvorlagen, Arbeitsprotokoll, Daily Note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
+++ b/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSacher\Desktop\Obsidian-Vault\02 Projekte\Bachelorarbeit\Testdurchläufe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BA8F25-A4C8-42C1-AFFB-8CB1EDBF48EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE4E544-C245-47F6-95DC-498D126C650A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anleitung" sheetId="1" r:id="rId1"/>
@@ -878,12 +878,12 @@
     <xf numFmtId="169" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="170" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1428,7 +1428,7 @@
       <c r="A8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="41">
+      <c r="B8" s="38">
         <v>256</v>
       </c>
       <c r="D8" s="9" t="s">
@@ -1667,11 +1667,11 @@
       <c r="A32" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="38" t="s">
+      <c r="B32" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="39"/>
-      <c r="D32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
BA: Session 20.10.2026 -- Vorab-Anfragen TF 4/5, Templates repariert und neu sortiert, Ablauf Testtag, Arbeitsprotokoll, Daily Note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
+++ b/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSacher\Desktop\Obsidian-Vault\02 Projekte\Bachelorarbeit\Testdurchläufe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE4E544-C245-47F6-95DC-498D126C650A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330E699E-A960-4938-A25B-D3F5A7CADBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12790" yWindow="3540" windowWidth="19360" windowHeight="9910" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anleitung" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="206">
   <si>
     <t>Protokoll Testdurchläufe AsiMiNu</t>
   </si>
@@ -659,6 +659,15 @@
 5. Datenqualität: nach jedem Durchlauf Feld für Feld Soll gegen Ist (Ist: Template bzw. Anfrage im System).
 6. Befragung: Antworten aus dem Fragebogen.
 7. Auswertung: rechnet alles für Abschnitt 6.3 zusammen.</t>
+  </si>
+  <si>
+    <t>AdHoc-Testinstanz lief mit. Erste Mail TF 4 ursprünglich steht dort auf „Offen“.</t>
+  </si>
+  <si>
+    <t>AdHoc-Testinstanz lief mit. Erste Mail TF 5 ursprünglich dort auf „Gesendet“ gesetzt (gilt als ins TSM übertragen).</t>
+  </si>
+  <si>
+    <t>Vorab-Anfrage TF 5 ursprünglich am 20.10. von Hand validiert und mit „An TEF übertragen“ übertragen, nicht über einen Übertragungslauf.</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1383,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="32">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>24</v>
@@ -1541,11 +1550,11 @@
       </c>
       <c r="B23" s="16">
         <f>WORKDAY($B$3,5)+TIME(8,0,0)</f>
-        <v>46321.333333333336</v>
+        <v>46322.333333333336</v>
       </c>
       <c r="C23" s="16">
         <f>WORKDAY($B$3,5)+TIME(9,0,0)</f>
-        <v>46321.375</v>
+        <v>46322.375</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>54</v>
@@ -1557,11 +1566,11 @@
       </c>
       <c r="B24" s="16">
         <f>WORKDAY($B$3,6)+TIME(8,0,0)</f>
-        <v>46322.333333333336</v>
+        <v>46323.333333333336</v>
       </c>
       <c r="C24" s="16">
         <f>WORKDAY($B$3,6)+TIME(9,0,0)</f>
-        <v>46322.375</v>
+        <v>46323.375</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>56</v>
@@ -1573,11 +1582,11 @@
       </c>
       <c r="B25" s="16">
         <f>WORKDAY($B$3,7)+TIME(8,0,0)</f>
-        <v>46323.333333333336</v>
+        <v>46324.333333333336</v>
       </c>
       <c r="C25" s="16">
         <f>WORKDAY($B$3,7)+TIME(9,0,0)</f>
-        <v>46323.375</v>
+        <v>46324.375</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>58</v>
@@ -2670,7 +2679,9 @@
       <c r="U9" s="18"/>
       <c r="V9" s="22"/>
       <c r="W9" s="22"/>
-      <c r="X9" s="18"/>
+      <c r="X9" s="18" t="s">
+        <v>203</v>
+      </c>
       <c r="Y9" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2742,7 +2753,9 @@
       <c r="U10" s="18"/>
       <c r="V10" s="22"/>
       <c r="W10" s="22"/>
-      <c r="X10" s="18"/>
+      <c r="X10" s="18" t="s">
+        <v>204</v>
+      </c>
       <c r="Y10" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2814,7 +2827,9 @@
       <c r="U11" s="18"/>
       <c r="V11" s="22"/>
       <c r="W11" s="22"/>
-      <c r="X11" s="18"/>
+      <c r="X11" s="18" t="s">
+        <v>205</v>
+      </c>
       <c r="Y11" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -8109,7 +8124,7 @@
       </c>
       <c r="E9" s="16">
         <f>Testdaten!$B$23</f>
-        <v>46321.333333333336</v>
+        <v>46322.333333333336</v>
       </c>
       <c r="F9" s="18"/>
       <c r="G9" s="18"/>
@@ -8131,7 +8146,7 @@
       </c>
       <c r="E10" s="16">
         <f>Testdaten!$C$23</f>
-        <v>46321.375</v>
+        <v>46322.375</v>
       </c>
       <c r="F10" s="18"/>
       <c r="G10" s="18"/>
@@ -8328,7 +8343,7 @@
       </c>
       <c r="E19" s="16">
         <f>Testdaten!$B$23</f>
-        <v>46321.333333333336</v>
+        <v>46322.333333333336</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
@@ -8350,7 +8365,7 @@
       </c>
       <c r="E20" s="16">
         <f>Testdaten!$C$23</f>
-        <v>46321.375</v>
+        <v>46322.375</v>
       </c>
       <c r="F20" s="18"/>
       <c r="G20" s="18"/>
@@ -8546,7 +8561,7 @@
       </c>
       <c r="E29" s="16">
         <f>Testdaten!$B$24</f>
-        <v>46322.333333333336</v>
+        <v>46323.333333333336</v>
       </c>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -8568,7 +8583,7 @@
       </c>
       <c r="E30" s="16">
         <f>Testdaten!$C$24</f>
-        <v>46322.375</v>
+        <v>46323.375</v>
       </c>
       <c r="F30" s="18"/>
       <c r="G30" s="18"/>
@@ -8764,7 +8779,7 @@
       </c>
       <c r="E39" s="16">
         <f>Testdaten!$B$24</f>
-        <v>46322.333333333336</v>
+        <v>46323.333333333336</v>
       </c>
       <c r="F39" s="18"/>
       <c r="G39" s="18"/>
@@ -8786,7 +8801,7 @@
       </c>
       <c r="E40" s="16">
         <f>Testdaten!$C$24</f>
-        <v>46322.375</v>
+        <v>46323.375</v>
       </c>
       <c r="F40" s="18"/>
       <c r="G40" s="18"/>
@@ -8982,7 +8997,7 @@
       </c>
       <c r="E49" s="16">
         <f>Testdaten!$B$25</f>
-        <v>46323.333333333336</v>
+        <v>46324.333333333336</v>
       </c>
       <c r="F49" s="18"/>
       <c r="G49" s="18"/>
@@ -9004,7 +9019,7 @@
       </c>
       <c r="E50" s="16">
         <f>Testdaten!$C$25</f>
-        <v>46323.375</v>
+        <v>46324.375</v>
       </c>
       <c r="F50" s="18"/>
       <c r="G50" s="18"/>
@@ -9200,7 +9215,7 @@
       </c>
       <c r="E59" s="16">
         <f>Testdaten!$B$25</f>
-        <v>46323.333333333336</v>
+        <v>46324.333333333336</v>
       </c>
       <c r="F59" s="18"/>
       <c r="G59" s="18"/>
@@ -9222,7 +9237,7 @@
       </c>
       <c r="E60" s="16">
         <f>Testdaten!$C$25</f>
-        <v>46323.375</v>
+        <v>46324.375</v>
       </c>
       <c r="F60" s="18"/>
       <c r="G60" s="18"/>
@@ -10735,7 +10750,7 @@
       </c>
       <c r="E129" s="16">
         <f>Testdaten!$B$23</f>
-        <v>46321.333333333336</v>
+        <v>46322.333333333336</v>
       </c>
       <c r="F129" s="18"/>
       <c r="G129" s="18"/>
@@ -10757,7 +10772,7 @@
       </c>
       <c r="E130" s="16">
         <f>Testdaten!$C$23</f>
-        <v>46321.375</v>
+        <v>46322.375</v>
       </c>
       <c r="F130" s="18"/>
       <c r="G130" s="18"/>
@@ -10954,7 +10969,7 @@
       </c>
       <c r="E139" s="16">
         <f>Testdaten!$B$23</f>
-        <v>46321.333333333336</v>
+        <v>46322.333333333336</v>
       </c>
       <c r="F139" s="18"/>
       <c r="G139" s="18"/>
@@ -10976,7 +10991,7 @@
       </c>
       <c r="E140" s="16">
         <f>Testdaten!$C$23</f>
-        <v>46321.375</v>
+        <v>46322.375</v>
       </c>
       <c r="F140" s="18"/>
       <c r="G140" s="18"/>
@@ -11172,7 +11187,7 @@
       </c>
       <c r="E149" s="16">
         <f>Testdaten!$B$24</f>
-        <v>46322.333333333336</v>
+        <v>46323.333333333336</v>
       </c>
       <c r="F149" s="18"/>
       <c r="G149" s="18"/>
@@ -11194,7 +11209,7 @@
       </c>
       <c r="E150" s="16">
         <f>Testdaten!$C$24</f>
-        <v>46322.375</v>
+        <v>46323.375</v>
       </c>
       <c r="F150" s="18"/>
       <c r="G150" s="18"/>
@@ -11390,7 +11405,7 @@
       </c>
       <c r="E159" s="16">
         <f>Testdaten!$B$24</f>
-        <v>46322.333333333336</v>
+        <v>46323.333333333336</v>
       </c>
       <c r="F159" s="18"/>
       <c r="G159" s="18"/>
@@ -11412,7 +11427,7 @@
       </c>
       <c r="E160" s="16">
         <f>Testdaten!$C$24</f>
-        <v>46322.375</v>
+        <v>46323.375</v>
       </c>
       <c r="F160" s="18"/>
       <c r="G160" s="18"/>
@@ -11608,7 +11623,7 @@
       </c>
       <c r="E169" s="16">
         <f>Testdaten!$B$25</f>
-        <v>46323.333333333336</v>
+        <v>46324.333333333336</v>
       </c>
       <c r="F169" s="18"/>
       <c r="G169" s="18"/>
@@ -11630,7 +11645,7 @@
       </c>
       <c r="E170" s="16">
         <f>Testdaten!$C$25</f>
-        <v>46323.375</v>
+        <v>46324.375</v>
       </c>
       <c r="F170" s="18"/>
       <c r="G170" s="18"/>
@@ -11826,7 +11841,7 @@
       </c>
       <c r="E179" s="16">
         <f>Testdaten!$B$25</f>
-        <v>46323.333333333336</v>
+        <v>46324.333333333336</v>
       </c>
       <c r="F179" s="18"/>
       <c r="G179" s="18"/>
@@ -11848,7 +11863,7 @@
       </c>
       <c r="E180" s="16">
         <f>Testdaten!$C$25</f>
-        <v>46323.375</v>
+        <v>46324.375</v>
       </c>
       <c r="F180" s="18"/>
       <c r="G180" s="18"/>

</xml_diff>

<commit_message>
BA: Protokoll Testdurchläufe (21.10.2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
+++ b/02 Projekte/Bachelorarbeit/Testdurchläufe/Protokoll Testdurchläufe.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSacher\Desktop\Obsidian-Vault\02 Projekte\Bachelorarbeit\Testdurchläufe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b7199ff5b15df6c/Desktop/Obsidian-Vault/02 Projekte/Bachelorarbeit/Testdurchläufe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330E699E-A960-4938-A25B-D3F5A7CADBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="13_ncr:1_{330E699E-A960-4938-A25B-D3F5A7CADBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8265A924-964E-4F35-89A4-1AC5D0CD629C}"/>
   <bookViews>
-    <workbookView xWindow="12790" yWindow="3540" windowWidth="19360" windowHeight="9910" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anleitung" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="212">
   <si>
     <t>Protokoll Testdurchläufe AsiMiNu</t>
   </si>
@@ -661,13 +661,31 @@
 7. Auswertung: rechnet alles für Abschnitt 6.3 zusammen.</t>
   </si>
   <si>
-    <t>AdHoc-Testinstanz lief mit. Erste Mail TF 4 ursprünglich steht dort auf „Offen“.</t>
-  </si>
-  <si>
-    <t>AdHoc-Testinstanz lief mit. Erste Mail TF 5 ursprünglich dort auf „Gesendet“ gesetzt (gilt als ins TSM übertragen).</t>
-  </si>
-  <si>
-    <t>Vorab-Anfrage TF 5 ursprünglich am 20.10. von Hand validiert und mit „An TEF übertragen“ übertragen, nicht über einen Übertragungslauf.</t>
+    <t>P2(DI)</t>
+  </si>
+  <si>
+    <t>P1(FE)</t>
+  </si>
+  <si>
+    <t>nein</t>
+  </si>
+  <si>
+    <t>Minimal 2 stunden und maximal kann eine woche</t>
+  </si>
+  <si>
+    <t>Das hat die App nicht gelesen</t>
+  </si>
+  <si>
+    <t>15-20 Minuten Tsm arbeit</t>
+  </si>
+  <si>
+    <t>15 sekunden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was, denke ich mal, für fast alle Testfälle gleich ist, ist, wie lange der GU ungefähr braucht, um die Daten in das Template zu schreiben. Das habe ich nämlich vorhin einmal getestet mit einer aus unserer Arbeit, die ich sozusagen GU spielen lassen habe. Sie hat ungefähr das Template eingetragen, bis zum Abschicken der E-Mail, also mit Betreffenden die E-Mail geschrieben und alles drum und dran, ungefähr. </t>
+  </si>
+  <si>
+    <t>GU</t>
   </si>
 </sst>
 </file>
@@ -683,7 +701,7 @@
     <numFmt numFmtId="169" formatCode="\d\d\.mm/\y\y\y\y"/>
     <numFmt numFmtId="170" formatCode="#,#00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -731,6 +749,12 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -908,6 +932,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2145,56 +2173,72 @@
       <c r="E2" s="14">
         <v>1</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20" t="str">
+      <c r="F2" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H2" s="8">
+        <v>46316</v>
+      </c>
+      <c r="I2" s="19">
+        <v>0.64594907407407409</v>
+      </c>
+      <c r="J2" s="19">
+        <v>0.6490393518518518</v>
+      </c>
+      <c r="K2" s="20">
         <f t="shared" ref="K2:K25" si="0">IF(OR(I2="",J2=""),"",ROUND((J2-I2)*1440,1))</f>
-        <v/>
-      </c>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="20" t="str">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="L2" s="19">
+        <v>0.65115740740740746</v>
+      </c>
+      <c r="M2" s="19">
+        <v>0.65127314814814818</v>
+      </c>
+      <c r="N2" s="20">
         <f t="shared" ref="N2:N25" si="1">IF(OR(L2="",M2=""),"",ROUND((M2-L2)*1440,1))</f>
-        <v/>
-      </c>
-      <c r="O2" s="18"/>
+        <v>0.2</v>
+      </c>
+      <c r="O2" s="18" t="s">
+        <v>205</v>
+      </c>
       <c r="P2" s="21"/>
-      <c r="Q2" s="20" t="str">
+      <c r="Q2" s="20">
         <f t="shared" ref="Q2:Q25" si="2">IF(K2="","",SUM(K2,N2,P2))</f>
-        <v/>
+        <v>4.6000000000000005</v>
       </c>
       <c r="R2" s="18"/>
       <c r="S2" s="18"/>
       <c r="T2" s="11" t="str">
         <f>IF(K2="","",IF(COUNTIFS(Fehler!$B$2:$B$200,A2,Fehler!$I$2:$I$200,"ja")&gt;0,"ja","nein"))</f>
-        <v/>
+        <v>nein</v>
       </c>
       <c r="U2" s="18"/>
       <c r="V2" s="22"/>
       <c r="W2" s="22"/>
       <c r="X2" s="18"/>
-      <c r="Y2" s="23" t="str">
+      <c r="Y2" s="23">
         <f t="shared" ref="Y2:Y25" si="3">IF(AND(D2="alt",K2&lt;&gt;""),K2,"")</f>
-        <v/>
+        <v>4.4000000000000004</v>
       </c>
       <c r="Z2" s="23" t="str">
         <f t="shared" ref="Z2:Z25" si="4">IF(AND(D2="neu",K2&lt;&gt;""),K2,"")</f>
         <v/>
       </c>
-      <c r="AA2" s="23" t="str">
+      <c r="AA2" s="23">
         <f t="shared" ref="AA2:AA25" si="5">IF(AND(D2="alt",K2&lt;&gt;""),SUM(N2,P2),"")</f>
-        <v/>
+        <v>0.2</v>
       </c>
       <c r="AB2" s="23" t="str">
         <f t="shared" ref="AB2:AB25" si="6">IF(AND(D2="neu",K2&lt;&gt;""),SUM(N2,P2),"")</f>
         <v/>
       </c>
-      <c r="AC2" s="23" t="str">
+      <c r="AC2" s="23">
         <f t="shared" ref="AC2:AC25" si="7">IF(AND(D2="alt",K2&lt;&gt;""),Q2,"")</f>
-        <v/>
+        <v>4.6000000000000005</v>
       </c>
       <c r="AD2" s="23" t="str">
         <f t="shared" ref="AD2:AD25" si="8">IF(AND(D2="neu",K2&lt;&gt;""),SUM(K2,N2,P2),"")</f>
@@ -2217,9 +2261,15 @@
       <c r="E3" s="14">
         <v>2</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="8"/>
+      <c r="F3" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H3" s="8">
+        <v>46316</v>
+      </c>
       <c r="I3" s="19"/>
       <c r="J3" s="19"/>
       <c r="K3" s="20" t="str">
@@ -2228,9 +2278,8 @@
       </c>
       <c r="L3" s="19"/>
       <c r="M3" s="19"/>
-      <c r="N3" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="N3" s="20">
+        <v>120</v>
       </c>
       <c r="O3" s="18"/>
       <c r="P3" s="21"/>
@@ -2247,7 +2296,9 @@
       <c r="U3" s="18"/>
       <c r="V3" s="22"/>
       <c r="W3" s="22"/>
-      <c r="X3" s="18"/>
+      <c r="X3" s="18" t="s">
+        <v>206</v>
+      </c>
       <c r="Y3" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2289,9 +2340,15 @@
       <c r="E4" s="14">
         <v>1</v>
       </c>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="8"/>
+      <c r="F4" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H4" s="8">
+        <v>46316</v>
+      </c>
       <c r="I4" s="19"/>
       <c r="J4" s="19"/>
       <c r="K4" s="20" t="str">
@@ -2300,14 +2357,10 @@
       </c>
       <c r="L4" s="19"/>
       <c r="M4" s="19"/>
-      <c r="N4" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
       <c r="O4" s="18"/>
       <c r="P4" s="21"/>
       <c r="Q4" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(K4="","",SUM(K4,N5,P4))</f>
         <v/>
       </c>
       <c r="R4" s="18"/>
@@ -2329,11 +2382,11 @@
         <v/>
       </c>
       <c r="AA4" s="23" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(AND(D4="alt",K4&lt;&gt;""),SUM(N5,P4),"")</f>
         <v/>
       </c>
       <c r="AB4" s="23" t="str">
-        <f t="shared" si="6"/>
+        <f>IF(AND(D4="neu",K4&lt;&gt;""),SUM(N5,P4),"")</f>
         <v/>
       </c>
       <c r="AC4" s="23" t="str">
@@ -2341,7 +2394,7 @@
         <v/>
       </c>
       <c r="AD4" s="23" t="str">
-        <f t="shared" si="8"/>
+        <f>IF(AND(D4="neu",K4&lt;&gt;""),SUM(K4,N5,P4),"")</f>
         <v/>
       </c>
     </row>
@@ -2361,9 +2414,15 @@
       <c r="E5" s="14">
         <v>2</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="8"/>
+      <c r="F5" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H5" s="8">
+        <v>46316</v>
+      </c>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
       <c r="K5" s="20" t="str">
@@ -2372,14 +2431,13 @@
       </c>
       <c r="L5" s="19"/>
       <c r="M5" s="19"/>
-      <c r="N5" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="N5" s="20">
+        <v>120</v>
       </c>
       <c r="O5" s="18"/>
       <c r="P5" s="21"/>
       <c r="Q5" s="20" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(K5="","",SUM(K5,#REF!,P5))</f>
         <v/>
       </c>
       <c r="R5" s="18"/>
@@ -2401,11 +2459,11 @@
         <v/>
       </c>
       <c r="AA5" s="23" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(AND(D5="alt",K5&lt;&gt;""),SUM(#REF!,P5),"")</f>
         <v/>
       </c>
       <c r="AB5" s="23" t="str">
-        <f t="shared" si="6"/>
+        <f>IF(AND(D5="neu",K5&lt;&gt;""),SUM(#REF!,P5),"")</f>
         <v/>
       </c>
       <c r="AC5" s="23" t="str">
@@ -2413,7 +2471,7 @@
         <v/>
       </c>
       <c r="AD5" s="23" t="str">
-        <f t="shared" si="8"/>
+        <f>IF(AND(D5="neu",K5&lt;&gt;""),SUM(K5,#REF!,P5),"")</f>
         <v/>
       </c>
     </row>
@@ -2433,9 +2491,15 @@
       <c r="E6" s="14">
         <v>1</v>
       </c>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="8"/>
+      <c r="F6" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H6" s="8">
+        <v>46316</v>
+      </c>
       <c r="I6" s="19"/>
       <c r="J6" s="19"/>
       <c r="K6" s="20" t="str">
@@ -2444,9 +2508,8 @@
       </c>
       <c r="L6" s="19"/>
       <c r="M6" s="19"/>
-      <c r="N6" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="N6" s="20">
+        <v>120</v>
       </c>
       <c r="O6" s="18"/>
       <c r="P6" s="21"/>
@@ -2505,9 +2568,15 @@
       <c r="E7" s="14">
         <v>2</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="8"/>
+      <c r="F7" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H7" s="8">
+        <v>46316</v>
+      </c>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
       <c r="K7" s="20" t="str">
@@ -2577,9 +2646,15 @@
       <c r="E8" s="14">
         <v>1</v>
       </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="8"/>
+      <c r="F8" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H8" s="8">
+        <v>46316</v>
+      </c>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
       <c r="K8" s="20" t="str">
@@ -2607,7 +2682,9 @@
       <c r="U8" s="18"/>
       <c r="V8" s="22"/>
       <c r="W8" s="22"/>
-      <c r="X8" s="18"/>
+      <c r="X8" s="18" t="s">
+        <v>207</v>
+      </c>
       <c r="Y8" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2649,9 +2726,15 @@
       <c r="E9" s="14">
         <v>2</v>
       </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="8"/>
+      <c r="F9" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H9" s="8">
+        <v>46316</v>
+      </c>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="20" t="str">
@@ -2679,9 +2762,7 @@
       <c r="U9" s="18"/>
       <c r="V9" s="22"/>
       <c r="W9" s="22"/>
-      <c r="X9" s="18" t="s">
-        <v>203</v>
-      </c>
+      <c r="X9" s="18"/>
       <c r="Y9" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2723,9 +2804,15 @@
       <c r="E10" s="14">
         <v>1</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="8"/>
+      <c r="F10" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H10" s="8">
+        <v>46316</v>
+      </c>
       <c r="I10" s="19"/>
       <c r="J10" s="19"/>
       <c r="K10" s="20" t="str">
@@ -2754,7 +2841,7 @@
       <c r="V10" s="22"/>
       <c r="W10" s="22"/>
       <c r="X10" s="18" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="Y10" s="23" t="str">
         <f t="shared" si="3"/>
@@ -2797,9 +2884,15 @@
       <c r="E11" s="14">
         <v>2</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="8"/>
+      <c r="F11" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H11" s="8">
+        <v>46316</v>
+      </c>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
       <c r="K11" s="20" t="str">
@@ -2808,9 +2901,8 @@
       </c>
       <c r="L11" s="19"/>
       <c r="M11" s="19"/>
-      <c r="N11" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="N11" s="20" t="s">
+        <v>210</v>
       </c>
       <c r="O11" s="18"/>
       <c r="P11" s="21"/>
@@ -2827,9 +2919,7 @@
       <c r="U11" s="18"/>
       <c r="V11" s="22"/>
       <c r="W11" s="22"/>
-      <c r="X11" s="18" t="s">
-        <v>205</v>
-      </c>
+      <c r="X11" s="18"/>
       <c r="Y11" s="23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2871,9 +2961,15 @@
       <c r="E12" s="14">
         <v>1</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="8"/>
+      <c r="F12" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H12" s="8">
+        <v>46316</v>
+      </c>
       <c r="I12" s="19"/>
       <c r="J12" s="19"/>
       <c r="K12" s="20" t="str">
@@ -2943,9 +3039,15 @@
       <c r="E13" s="14">
         <v>2</v>
       </c>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="8"/>
+      <c r="F13" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H13" s="8">
+        <v>46316</v>
+      </c>
       <c r="I13" s="19"/>
       <c r="J13" s="19"/>
       <c r="K13" s="20" t="str">
@@ -2954,9 +3056,8 @@
       </c>
       <c r="L13" s="19"/>
       <c r="M13" s="19"/>
-      <c r="N13" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="N13" s="20" t="s">
+        <v>209</v>
       </c>
       <c r="O13" s="18"/>
       <c r="P13" s="21"/>
@@ -3864,6 +3965,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" error="Bitte einen Wert aus der Liste wählen." sqref="R2:R25" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"übertragen,vorgemerkt (Automatik),manuelle Prüfung,abgelehnt,verworfen,abgebrochen"</formula1>
@@ -3876,6 +3978,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13260,14 +13363,18 @@
       <c r="A2" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="18"/>
+      <c r="B2" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C2" s="14">
         <v>1</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="E2" s="18"/>
+      <c r="E2" s="18">
+        <v>5</v>
+      </c>
       <c r="F2" s="18"/>
       <c r="G2" s="18"/>
     </row>
@@ -13275,14 +13382,18 @@
       <c r="A3" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="18"/>
+      <c r="B3" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C3" s="14">
         <v>2</v>
       </c>
       <c r="D3" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="18"/>
+      <c r="E3" s="18">
+        <v>5</v>
+      </c>
       <c r="F3" s="18"/>
       <c r="G3" s="18"/>
     </row>
@@ -13290,14 +13401,18 @@
       <c r="A4" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="18"/>
+      <c r="B4" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C4" s="14">
         <v>3</v>
       </c>
       <c r="D4" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="E4" s="18"/>
+      <c r="E4" s="18">
+        <v>5</v>
+      </c>
       <c r="F4" s="18"/>
       <c r="G4" s="18"/>
     </row>
@@ -13305,7 +13420,9 @@
       <c r="A5" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B5" s="18"/>
+      <c r="B5" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C5" s="14">
         <v>4</v>
       </c>
@@ -13320,7 +13437,9 @@
       <c r="A6" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="18"/>
+      <c r="B6" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C6" s="14">
         <v>5</v>
       </c>
@@ -13335,7 +13454,9 @@
       <c r="A7" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="18"/>
+      <c r="B7" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C7" s="14">
         <v>6</v>
       </c>
@@ -13350,7 +13471,9 @@
       <c r="A8" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="18"/>
+      <c r="B8" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C8" s="14">
         <v>7</v>
       </c>
@@ -13365,7 +13488,9 @@
       <c r="A9" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="18"/>
+      <c r="B9" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C9" s="14">
         <v>8</v>
       </c>
@@ -13722,7 +13847,9 @@
       <c r="A32" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="18"/>
+      <c r="B32" s="18" t="s">
+        <v>211</v>
+      </c>
       <c r="C32" s="14">
         <v>7</v>
       </c>
@@ -14072,9 +14199,9 @@
       <c r="A6" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="20" t="str">
+      <c r="B6" s="20">
         <f>IFERROR(MEDIAN(Durchläufe!$Y$2:$Y$25),"–")</f>
-        <v>–</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="C6" s="20" t="str">
         <f>IFERROR(MEDIAN(Durchläufe!$Z$2:$Z$25),"–")</f>
@@ -14093,9 +14220,9 @@
       <c r="A7" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="20" t="str">
+      <c r="B7" s="20">
         <f>IFERROR(MEDIAN(Durchläufe!$AA$2:$AA$25),"–")</f>
-        <v>–</v>
+        <v>0.2</v>
       </c>
       <c r="C7" s="20" t="str">
         <f>IFERROR(MEDIAN(Durchläufe!$AB$2:$AB$25),"–")</f>
@@ -14137,9 +14264,9 @@
       <c r="A9" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B9" s="28" t="str">
+      <c r="B9" s="28">
         <f>IFERROR(MEDIAN(Durchläufe!$AC$2:$AC$25)+IF(ISNUMBER(B8),B8,0),"–")</f>
-        <v>–</v>
+        <v>4.6000000000000005</v>
       </c>
       <c r="C9" s="28" t="str">
         <f>IFERROR(MEDIAN(Durchläufe!$AD$2:$AD$25),"–")</f>
@@ -14160,7 +14287,7 @@
       </c>
       <c r="B10" s="11">
         <f>COUNT(Durchläufe!$AC$2:$AC$25)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" s="11">
         <f>COUNT(Durchläufe!$AD$2:$AD$25)</f>
@@ -14206,9 +14333,9 @@
       <c r="A14" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="29" t="str">
+      <c r="B14" s="29">
         <f>IFERROR(COUNTIFS(Durchläufe!$D$2:$D$25,"alt",Durchläufe!$T$2:$T$25,"ja")/(COUNTIFS(Durchläufe!$D$2:$D$25,"alt",Durchläufe!$T$2:$T$25,"ja")+COUNTIFS(Durchläufe!$D$2:$D$25,"alt",Durchläufe!$T$2:$T$25,"nein")),"–")</f>
-        <v>–</v>
+        <v>0</v>
       </c>
       <c r="C14" s="29" t="str">
         <f>IFERROR(COUNTIFS(Durchläufe!$D$2:$D$25,"neu",Durchläufe!$T$2:$T$25,"ja")/(COUNTIFS(Durchläufe!$D$2:$D$25,"neu",Durchläufe!$T$2:$T$25,"ja")+COUNTIFS(Durchläufe!$D$2:$D$25,"neu",Durchläufe!$T$2:$T$25,"nein")),"–")</f>
@@ -14394,9 +14521,9 @@
       <c r="A33" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="B33" s="20" t="str">
+      <c r="B33" s="20">
         <f>IFERROR(AVERAGEIFS(Befragung!$E$2:$E$49,Befragung!$C$2:$C$49,1),"–")</f>
-        <v>–</v>
+        <v>5</v>
       </c>
       <c r="C33" s="20" t="str">
         <f>IFERROR(AVERAGEIFS(Befragung!$F$2:$F$49,Befragung!$C$2:$C$49,1),"–")</f>
@@ -14407,9 +14534,9 @@
       <c r="A34" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="B34" s="20" t="str">
+      <c r="B34" s="20">
         <f>IFERROR(AVERAGEIFS(Befragung!$E$2:$E$49,Befragung!$C$2:$C$49,2),"–")</f>
-        <v>–</v>
+        <v>5</v>
       </c>
       <c r="C34" s="20" t="str">
         <f>IFERROR(AVERAGEIFS(Befragung!$F$2:$F$49,Befragung!$C$2:$C$49,2),"–")</f>
@@ -14420,9 +14547,9 @@
       <c r="A35" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="B35" s="20" t="str">
+      <c r="B35" s="20">
         <f>IFERROR(AVERAGEIFS(Befragung!$E$2:$E$49,Befragung!$C$2:$C$49,3),"–")</f>
-        <v>–</v>
+        <v>5</v>
       </c>
       <c r="C35" s="20" t="str">
         <f>IFERROR(AVERAGEIFS(Befragung!$F$2:$F$49,Befragung!$C$2:$C$49,3),"–")</f>

</xml_diff>